<commit_message>
Use the store's Trendyol brand ixoskids club for the Minah Tekstil upload
"Minah Tekstil" is the seller name, not a brand Trendyol knows; the
store's existing products are listed under the ixoskids club brand.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJxz6TxayURknP2UowWRAx
</commit_message>
<xml_diff>
--- a/minah-tekstil/trendyol/minah-trendyol-dosya-1.xlsx
+++ b/minah-tekstil/trendyol/minah-trendyol-dosya-1.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8129" uniqueCount="3420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8129" uniqueCount="3421">
   <si>
     <t>Barkod</t>
   </si>
@@ -10256,6 +10256,9 @@
   </si>
   <si>
     <t>MNH-TAYT</t>
+  </si>
+  <si>
+    <t>ixoskids club</t>
   </si>
   <si>
     <t xml:space="preserve">Detaylar: Yüksek bel, uzun paça, vücuda oturan kesim, melanj görünüm
@@ -11568,7 +11571,7 @@
         <v>3327</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D2" t="s">
         <v>69</v>
@@ -11580,7 +11583,7 @@
         <v>235</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3328</v>
+        <v>3329</v>
       </c>
       <c r="H2" s="38">
         <v>650</v>
@@ -11645,13 +11648,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3329</v>
+        <v>3330</v>
       </c>
       <c r="B3" t="s">
         <v>3327</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D3" t="s">
         <v>69</v>
@@ -11663,7 +11666,7 @@
         <v>235</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3328</v>
+        <v>3329</v>
       </c>
       <c r="H3" s="38">
         <v>650</v>
@@ -11675,7 +11678,7 @@
         <v>6</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3329</v>
+        <v>3330</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -11728,13 +11731,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3330</v>
+        <v>3331</v>
       </c>
       <c r="B4" t="s">
         <v>3327</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D4" t="s">
         <v>69</v>
@@ -11746,7 +11749,7 @@
         <v>235</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3328</v>
+        <v>3329</v>
       </c>
       <c r="H4" s="38">
         <v>650</v>
@@ -11758,7 +11761,7 @@
         <v>6</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3330</v>
+        <v>3331</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -11811,13 +11814,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3331</v>
+        <v>3332</v>
       </c>
       <c r="B5" t="s">
         <v>3327</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D5" t="s">
         <v>69</v>
@@ -11829,7 +11832,7 @@
         <v>235</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3328</v>
+        <v>3329</v>
       </c>
       <c r="H5" s="38">
         <v>650</v>
@@ -11841,7 +11844,7 @@
         <v>6</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3331</v>
+        <v>3332</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -11894,13 +11897,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3332</v>
+        <v>3333</v>
       </c>
       <c r="B6" t="s">
         <v>3327</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D6" t="s">
         <v>69</v>
@@ -11912,7 +11915,7 @@
         <v>251</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="H6" s="38">
         <v>650</v>
@@ -11924,7 +11927,7 @@
         <v>6</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3332</v>
+        <v>3333</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -11971,13 +11974,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>3334</v>
+        <v>3335</v>
       </c>
       <c r="B7" t="s">
         <v>3327</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D7" t="s">
         <v>69</v>
@@ -11989,7 +11992,7 @@
         <v>251</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="H7" s="38">
         <v>650</v>
@@ -12001,7 +12004,7 @@
         <v>6</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3334</v>
+        <v>3335</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -12048,13 +12051,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3335</v>
+        <v>3336</v>
       </c>
       <c r="B8" t="s">
         <v>3327</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D8" t="s">
         <v>69</v>
@@ -12066,7 +12069,7 @@
         <v>251</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="H8" s="38">
         <v>650</v>
@@ -12078,7 +12081,7 @@
         <v>6</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3335</v>
+        <v>3336</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -12125,13 +12128,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>3336</v>
+        <v>3337</v>
       </c>
       <c r="B9" t="s">
         <v>3327</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D9" t="s">
         <v>69</v>
@@ -12143,7 +12146,7 @@
         <v>251</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="H9" s="38">
         <v>650</v>
@@ -12155,7 +12158,7 @@
         <v>6</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3336</v>
+        <v>3337</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -15505,13 +15508,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3400</v>
+        <v>3401</v>
       </c>
       <c r="B2" t="s">
-        <v>3401</v>
+        <v>3402</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D2" t="s">
         <v>370</v>
@@ -15520,10 +15523,10 @@
         <v>70</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>3402</v>
+        <v>3403</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3403</v>
+        <v>3404</v>
       </c>
       <c r="H2" s="38">
         <v>1000</v>
@@ -15535,7 +15538,7 @@
         <v>2</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3400</v>
+        <v>3401</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -15582,13 +15585,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3404</v>
+        <v>3405</v>
       </c>
       <c r="B3" t="s">
-        <v>3401</v>
+        <v>3402</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D3" t="s">
         <v>370</v>
@@ -15597,10 +15600,10 @@
         <v>70</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>3402</v>
+        <v>3403</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3403</v>
+        <v>3404</v>
       </c>
       <c r="H3" s="38">
         <v>1000</v>
@@ -15612,7 +15615,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3404</v>
+        <v>3405</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -15659,13 +15662,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3405</v>
+        <v>3406</v>
       </c>
       <c r="B4" t="s">
-        <v>3401</v>
+        <v>3402</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D4" t="s">
         <v>370</v>
@@ -15674,10 +15677,10 @@
         <v>70</v>
       </c>
       <c r="F4" s="35" t="s">
-        <v>3402</v>
+        <v>3403</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3403</v>
+        <v>3404</v>
       </c>
       <c r="H4" s="38">
         <v>1000</v>
@@ -15689,7 +15692,7 @@
         <v>2</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3405</v>
+        <v>3406</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -15736,13 +15739,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3406</v>
+        <v>3407</v>
       </c>
       <c r="B5" t="s">
-        <v>3401</v>
+        <v>3402</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D5" t="s">
         <v>370</v>
@@ -15751,10 +15754,10 @@
         <v>70</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>3402</v>
+        <v>3403</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3403</v>
+        <v>3404</v>
       </c>
       <c r="H5" s="38">
         <v>1000</v>
@@ -15766,7 +15769,7 @@
         <v>2</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3406</v>
+        <v>3407</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -15813,13 +15816,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3407</v>
+        <v>3408</v>
       </c>
       <c r="B6" t="s">
-        <v>3408</v>
+        <v>3409</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D6" t="s">
         <v>370</v>
@@ -15828,10 +15831,10 @@
         <v>70</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>3409</v>
+        <v>3410</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3410</v>
+        <v>3411</v>
       </c>
       <c r="H6" s="38">
         <v>850</v>
@@ -15843,7 +15846,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3407</v>
+        <v>3408</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -15890,13 +15893,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>3411</v>
+        <v>3412</v>
       </c>
       <c r="B7" t="s">
-        <v>3408</v>
+        <v>3409</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D7" t="s">
         <v>370</v>
@@ -15905,10 +15908,10 @@
         <v>70</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>3409</v>
+        <v>3410</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3410</v>
+        <v>3411</v>
       </c>
       <c r="H7" s="38">
         <v>850</v>
@@ -15920,7 +15923,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3411</v>
+        <v>3412</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -15967,13 +15970,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3412</v>
+        <v>3413</v>
       </c>
       <c r="B8" t="s">
-        <v>3408</v>
+        <v>3409</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D8" t="s">
         <v>370</v>
@@ -15982,10 +15985,10 @@
         <v>70</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>3409</v>
+        <v>3410</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3410</v>
+        <v>3411</v>
       </c>
       <c r="H8" s="38">
         <v>850</v>
@@ -15997,7 +16000,7 @@
         <v>1</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3412</v>
+        <v>3413</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -16044,13 +16047,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>3413</v>
+        <v>3414</v>
       </c>
       <c r="B9" t="s">
-        <v>3408</v>
+        <v>3409</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D9" t="s">
         <v>370</v>
@@ -16059,10 +16062,10 @@
         <v>70</v>
       </c>
       <c r="F9" s="35" t="s">
-        <v>3409</v>
+        <v>3410</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3410</v>
+        <v>3411</v>
       </c>
       <c r="H9" s="38">
         <v>850</v>
@@ -16074,7 +16077,7 @@
         <v>1</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3413</v>
+        <v>3414</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -16121,13 +16124,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>3414</v>
+        <v>3415</v>
       </c>
       <c r="B10" t="s">
-        <v>3408</v>
+        <v>3409</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D10" t="s">
         <v>370</v>
@@ -16136,10 +16139,10 @@
         <v>70</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>3415</v>
+        <v>3416</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>3416</v>
+        <v>3417</v>
       </c>
       <c r="H10" s="38">
         <v>850</v>
@@ -16151,7 +16154,7 @@
         <v>1</v>
       </c>
       <c r="K10" s="39" t="s">
-        <v>3414</v>
+        <v>3415</v>
       </c>
       <c r="L10" s="39">
         <v>10</v>
@@ -16198,13 +16201,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>3417</v>
+        <v>3418</v>
       </c>
       <c r="B11" t="s">
-        <v>3408</v>
+        <v>3409</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D11" t="s">
         <v>370</v>
@@ -16213,10 +16216,10 @@
         <v>70</v>
       </c>
       <c r="F11" s="35" t="s">
-        <v>3415</v>
+        <v>3416</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>3416</v>
+        <v>3417</v>
       </c>
       <c r="H11" s="38">
         <v>850</v>
@@ -16228,7 +16231,7 @@
         <v>1</v>
       </c>
       <c r="K11" s="39" t="s">
-        <v>3417</v>
+        <v>3418</v>
       </c>
       <c r="L11" s="39">
         <v>10</v>
@@ -16275,13 +16278,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>3418</v>
+        <v>3419</v>
       </c>
       <c r="B12" t="s">
-        <v>3408</v>
+        <v>3409</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D12" t="s">
         <v>370</v>
@@ -16290,10 +16293,10 @@
         <v>70</v>
       </c>
       <c r="F12" s="35" t="s">
-        <v>3415</v>
+        <v>3416</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>3416</v>
+        <v>3417</v>
       </c>
       <c r="H12" s="38">
         <v>850</v>
@@ -16305,7 +16308,7 @@
         <v>1</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>3418</v>
+        <v>3419</v>
       </c>
       <c r="L12" s="39">
         <v>10</v>
@@ -16352,13 +16355,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>3419</v>
+        <v>3420</v>
       </c>
       <c r="B13" t="s">
-        <v>3408</v>
+        <v>3409</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D13" t="s">
         <v>370</v>
@@ -16367,10 +16370,10 @@
         <v>70</v>
       </c>
       <c r="F13" s="35" t="s">
-        <v>3415</v>
+        <v>3416</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>3416</v>
+        <v>3417</v>
       </c>
       <c r="H13" s="38">
         <v>850</v>
@@ -16382,7 +16385,7 @@
         <v>1</v>
       </c>
       <c r="K13" s="39" t="s">
-        <v>3419</v>
+        <v>3420</v>
       </c>
       <c r="L13" s="39">
         <v>10</v>
@@ -54063,13 +54066,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="B2" t="s">
-        <v>3338</v>
+        <v>3339</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D2" t="s">
         <v>1653</v>
@@ -54078,10 +54081,10 @@
         <v>70</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>3339</v>
+        <v>3340</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3340</v>
+        <v>3341</v>
       </c>
       <c r="H2" s="38">
         <v>1700</v>
@@ -54093,7 +54096,7 @@
         <v>3</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -54143,13 +54146,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3341</v>
+        <v>3342</v>
       </c>
       <c r="B3" t="s">
-        <v>3338</v>
+        <v>3339</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D3" t="s">
         <v>1653</v>
@@ -54158,10 +54161,10 @@
         <v>70</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>3339</v>
+        <v>3340</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3340</v>
+        <v>3341</v>
       </c>
       <c r="H3" s="38">
         <v>1700</v>
@@ -54173,7 +54176,7 @@
         <v>3</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3341</v>
+        <v>3342</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -54223,13 +54226,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3342</v>
+        <v>3343</v>
       </c>
       <c r="B4" t="s">
-        <v>3338</v>
+        <v>3339</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D4" t="s">
         <v>1653</v>
@@ -54238,10 +54241,10 @@
         <v>70</v>
       </c>
       <c r="F4" s="35" t="s">
-        <v>3339</v>
+        <v>3340</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3340</v>
+        <v>3341</v>
       </c>
       <c r="H4" s="38">
         <v>1700</v>
@@ -54253,7 +54256,7 @@
         <v>3</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3342</v>
+        <v>3343</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -54303,13 +54306,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3343</v>
+        <v>3344</v>
       </c>
       <c r="B5" t="s">
-        <v>3338</v>
+        <v>3339</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D5" t="s">
         <v>1653</v>
@@ -54318,10 +54321,10 @@
         <v>70</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>3339</v>
+        <v>3340</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3340</v>
+        <v>3341</v>
       </c>
       <c r="H5" s="38">
         <v>1700</v>
@@ -54333,7 +54336,7 @@
         <v>3</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3343</v>
+        <v>3344</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -57673,13 +57676,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3344</v>
+        <v>3345</v>
       </c>
       <c r="B2" t="s">
-        <v>3345</v>
+        <v>3346</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D2" t="s">
         <v>355</v>
@@ -57688,10 +57691,10 @@
         <v>70</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>3346</v>
+        <v>3347</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3347</v>
+        <v>3348</v>
       </c>
       <c r="H2" s="38">
         <v>1100</v>
@@ -57703,7 +57706,7 @@
         <v>1</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3344</v>
+        <v>3345</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -57753,13 +57756,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3348</v>
+        <v>3349</v>
       </c>
       <c r="B3" t="s">
-        <v>3345</v>
+        <v>3346</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D3" t="s">
         <v>355</v>
@@ -57768,10 +57771,10 @@
         <v>70</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>3346</v>
+        <v>3347</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3347</v>
+        <v>3348</v>
       </c>
       <c r="H3" s="38">
         <v>1100</v>
@@ -57783,7 +57786,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3348</v>
+        <v>3349</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -57833,13 +57836,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3349</v>
+        <v>3350</v>
       </c>
       <c r="B4" t="s">
-        <v>3345</v>
+        <v>3346</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D4" t="s">
         <v>355</v>
@@ -57848,10 +57851,10 @@
         <v>70</v>
       </c>
       <c r="F4" s="35" t="s">
-        <v>3346</v>
+        <v>3347</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3347</v>
+        <v>3348</v>
       </c>
       <c r="H4" s="38">
         <v>1100</v>
@@ -57863,7 +57866,7 @@
         <v>1</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3349</v>
+        <v>3350</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -57913,13 +57916,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3350</v>
+        <v>3351</v>
       </c>
       <c r="B5" t="s">
-        <v>3345</v>
+        <v>3346</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D5" t="s">
         <v>355</v>
@@ -57928,10 +57931,10 @@
         <v>70</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>3346</v>
+        <v>3347</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3347</v>
+        <v>3348</v>
       </c>
       <c r="H5" s="38">
         <v>1100</v>
@@ -57943,7 +57946,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3350</v>
+        <v>3351</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -57993,13 +57996,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3351</v>
+        <v>3352</v>
       </c>
       <c r="B6" t="s">
-        <v>3345</v>
+        <v>3346</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D6" t="s">
         <v>355</v>
@@ -58008,10 +58011,10 @@
         <v>70</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>3346</v>
+        <v>3347</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3347</v>
+        <v>3348</v>
       </c>
       <c r="H6" s="38">
         <v>1100</v>
@@ -58023,7 +58026,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3351</v>
+        <v>3352</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -58073,13 +58076,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>3352</v>
+        <v>3353</v>
       </c>
       <c r="B7" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D7" t="s">
         <v>355</v>
@@ -58088,10 +58091,10 @@
         <v>70</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>3354</v>
+        <v>3355</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3355</v>
+        <v>3356</v>
       </c>
       <c r="H7" s="38">
         <v>1100</v>
@@ -58103,7 +58106,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3352</v>
+        <v>3353</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -58156,13 +58159,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3356</v>
+        <v>3357</v>
       </c>
       <c r="B8" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D8" t="s">
         <v>355</v>
@@ -58171,10 +58174,10 @@
         <v>70</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>3354</v>
+        <v>3355</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3355</v>
+        <v>3356</v>
       </c>
       <c r="H8" s="38">
         <v>1100</v>
@@ -58186,7 +58189,7 @@
         <v>1</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3356</v>
+        <v>3357</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -58239,13 +58242,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>3357</v>
+        <v>3358</v>
       </c>
       <c r="B9" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D9" t="s">
         <v>355</v>
@@ -58254,10 +58257,10 @@
         <v>70</v>
       </c>
       <c r="F9" s="35" t="s">
-        <v>3354</v>
+        <v>3355</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3355</v>
+        <v>3356</v>
       </c>
       <c r="H9" s="38">
         <v>1100</v>
@@ -58269,7 +58272,7 @@
         <v>1</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3357</v>
+        <v>3358</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -58322,13 +58325,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>3358</v>
+        <v>3359</v>
       </c>
       <c r="B10" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D10" t="s">
         <v>355</v>
@@ -58337,10 +58340,10 @@
         <v>70</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>3354</v>
+        <v>3355</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>3355</v>
+        <v>3356</v>
       </c>
       <c r="H10" s="38">
         <v>1100</v>
@@ -58352,7 +58355,7 @@
         <v>1</v>
       </c>
       <c r="K10" s="39" t="s">
-        <v>3358</v>
+        <v>3359</v>
       </c>
       <c r="L10" s="39">
         <v>10</v>
@@ -58405,13 +58408,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>3359</v>
+        <v>3360</v>
       </c>
       <c r="B11" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D11" t="s">
         <v>355</v>
@@ -58420,10 +58423,10 @@
         <v>70</v>
       </c>
       <c r="F11" s="35" t="s">
-        <v>3354</v>
+        <v>3355</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>3355</v>
+        <v>3356</v>
       </c>
       <c r="H11" s="38">
         <v>1100</v>
@@ -58435,7 +58438,7 @@
         <v>1</v>
       </c>
       <c r="K11" s="39" t="s">
-        <v>3359</v>
+        <v>3360</v>
       </c>
       <c r="L11" s="39">
         <v>10</v>
@@ -58488,13 +58491,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>3360</v>
+        <v>3361</v>
       </c>
       <c r="B12" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D12" t="s">
         <v>355</v>
@@ -58503,10 +58506,10 @@
         <v>70</v>
       </c>
       <c r="F12" s="35" t="s">
-        <v>3361</v>
+        <v>3362</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>3362</v>
+        <v>3363</v>
       </c>
       <c r="H12" s="38">
         <v>1100</v>
@@ -58518,7 +58521,7 @@
         <v>1</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>3360</v>
+        <v>3361</v>
       </c>
       <c r="L12" s="39">
         <v>10</v>
@@ -58568,13 +58571,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>3363</v>
+        <v>3364</v>
       </c>
       <c r="B13" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D13" t="s">
         <v>355</v>
@@ -58583,10 +58586,10 @@
         <v>70</v>
       </c>
       <c r="F13" s="35" t="s">
-        <v>3361</v>
+        <v>3362</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>3362</v>
+        <v>3363</v>
       </c>
       <c r="H13" s="38">
         <v>1100</v>
@@ -58598,7 +58601,7 @@
         <v>1</v>
       </c>
       <c r="K13" s="39" t="s">
-        <v>3363</v>
+        <v>3364</v>
       </c>
       <c r="L13" s="39">
         <v>10</v>
@@ -58648,13 +58651,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>3364</v>
+        <v>3365</v>
       </c>
       <c r="B14" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D14" t="s">
         <v>355</v>
@@ -58663,10 +58666,10 @@
         <v>70</v>
       </c>
       <c r="F14" s="35" t="s">
-        <v>3361</v>
+        <v>3362</v>
       </c>
       <c r="G14" s="35" t="s">
-        <v>3362</v>
+        <v>3363</v>
       </c>
       <c r="H14" s="38">
         <v>1100</v>
@@ -58678,7 +58681,7 @@
         <v>1</v>
       </c>
       <c r="K14" s="39" t="s">
-        <v>3364</v>
+        <v>3365</v>
       </c>
       <c r="L14" s="39">
         <v>10</v>
@@ -58728,13 +58731,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>3365</v>
+        <v>3366</v>
       </c>
       <c r="B15" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D15" t="s">
         <v>355</v>
@@ -58743,10 +58746,10 @@
         <v>70</v>
       </c>
       <c r="F15" s="35" t="s">
-        <v>3361</v>
+        <v>3362</v>
       </c>
       <c r="G15" s="35" t="s">
-        <v>3362</v>
+        <v>3363</v>
       </c>
       <c r="H15" s="38">
         <v>1100</v>
@@ -58758,7 +58761,7 @@
         <v>1</v>
       </c>
       <c r="K15" s="39" t="s">
-        <v>3365</v>
+        <v>3366</v>
       </c>
       <c r="L15" s="39">
         <v>10</v>
@@ -58808,13 +58811,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>3366</v>
+        <v>3367</v>
       </c>
       <c r="B16" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="C16" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D16" t="s">
         <v>355</v>
@@ -58823,10 +58826,10 @@
         <v>70</v>
       </c>
       <c r="F16" s="35" t="s">
-        <v>3361</v>
+        <v>3362</v>
       </c>
       <c r="G16" s="35" t="s">
-        <v>3362</v>
+        <v>3363</v>
       </c>
       <c r="H16" s="38">
         <v>1100</v>
@@ -58838,7 +58841,7 @@
         <v>1</v>
       </c>
       <c r="K16" s="39" t="s">
-        <v>3366</v>
+        <v>3367</v>
       </c>
       <c r="L16" s="39">
         <v>10</v>
@@ -58888,13 +58891,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>3367</v>
+        <v>3368</v>
       </c>
       <c r="B17" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D17" t="s">
         <v>355</v>
@@ -58903,10 +58906,10 @@
         <v>70</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>3369</v>
+        <v>3370</v>
       </c>
       <c r="G17" s="35" t="s">
-        <v>3370</v>
+        <v>3371</v>
       </c>
       <c r="H17" s="38">
         <v>1000</v>
@@ -58918,7 +58921,7 @@
         <v>1</v>
       </c>
       <c r="K17" s="39" t="s">
-        <v>3367</v>
+        <v>3368</v>
       </c>
       <c r="L17" s="39">
         <v>10</v>
@@ -58971,13 +58974,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>3371</v>
+        <v>3372</v>
       </c>
       <c r="B18" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D18" t="s">
         <v>355</v>
@@ -58986,10 +58989,10 @@
         <v>70</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>3369</v>
+        <v>3370</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>3370</v>
+        <v>3371</v>
       </c>
       <c r="H18" s="38">
         <v>1000</v>
@@ -59001,7 +59004,7 @@
         <v>1</v>
       </c>
       <c r="K18" s="39" t="s">
-        <v>3371</v>
+        <v>3372</v>
       </c>
       <c r="L18" s="39">
         <v>10</v>
@@ -59054,13 +59057,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>3372</v>
+        <v>3373</v>
       </c>
       <c r="B19" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D19" t="s">
         <v>355</v>
@@ -59069,10 +59072,10 @@
         <v>70</v>
       </c>
       <c r="F19" s="35" t="s">
-        <v>3369</v>
+        <v>3370</v>
       </c>
       <c r="G19" s="35" t="s">
-        <v>3370</v>
+        <v>3371</v>
       </c>
       <c r="H19" s="38">
         <v>1000</v>
@@ -59084,7 +59087,7 @@
         <v>1</v>
       </c>
       <c r="K19" s="39" t="s">
-        <v>3372</v>
+        <v>3373</v>
       </c>
       <c r="L19" s="39">
         <v>10</v>
@@ -59137,13 +59140,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>3373</v>
+        <v>3374</v>
       </c>
       <c r="B20" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D20" t="s">
         <v>355</v>
@@ -59152,10 +59155,10 @@
         <v>70</v>
       </c>
       <c r="F20" s="35" t="s">
-        <v>3369</v>
+        <v>3370</v>
       </c>
       <c r="G20" s="35" t="s">
-        <v>3370</v>
+        <v>3371</v>
       </c>
       <c r="H20" s="38">
         <v>1000</v>
@@ -59167,7 +59170,7 @@
         <v>1</v>
       </c>
       <c r="K20" s="39" t="s">
-        <v>3373</v>
+        <v>3374</v>
       </c>
       <c r="L20" s="39">
         <v>10</v>
@@ -59220,13 +59223,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>3374</v>
+        <v>3375</v>
       </c>
       <c r="B21" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D21" t="s">
         <v>355</v>
@@ -59235,10 +59238,10 @@
         <v>70</v>
       </c>
       <c r="F21" s="35" t="s">
-        <v>3369</v>
+        <v>3370</v>
       </c>
       <c r="G21" s="35" t="s">
-        <v>3370</v>
+        <v>3371</v>
       </c>
       <c r="H21" s="38">
         <v>1000</v>
@@ -59250,7 +59253,7 @@
         <v>1</v>
       </c>
       <c r="K21" s="39" t="s">
-        <v>3374</v>
+        <v>3375</v>
       </c>
       <c r="L21" s="39">
         <v>10</v>
@@ -59303,13 +59306,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>3375</v>
+        <v>3376</v>
       </c>
       <c r="B22" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C22" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D22" t="s">
         <v>355</v>
@@ -59318,10 +59321,10 @@
         <v>70</v>
       </c>
       <c r="F22" s="35" t="s">
-        <v>3376</v>
+        <v>3377</v>
       </c>
       <c r="G22" s="35" t="s">
-        <v>3377</v>
+        <v>3378</v>
       </c>
       <c r="H22" s="38">
         <v>1000</v>
@@ -59333,7 +59336,7 @@
         <v>1</v>
       </c>
       <c r="K22" s="39" t="s">
-        <v>3375</v>
+        <v>3376</v>
       </c>
       <c r="L22" s="39">
         <v>10</v>
@@ -59386,13 +59389,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>3378</v>
+        <v>3379</v>
       </c>
       <c r="B23" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D23" t="s">
         <v>355</v>
@@ -59401,10 +59404,10 @@
         <v>70</v>
       </c>
       <c r="F23" s="35" t="s">
-        <v>3376</v>
+        <v>3377</v>
       </c>
       <c r="G23" s="35" t="s">
-        <v>3377</v>
+        <v>3378</v>
       </c>
       <c r="H23" s="38">
         <v>1000</v>
@@ -59416,7 +59419,7 @@
         <v>1</v>
       </c>
       <c r="K23" s="39" t="s">
-        <v>3378</v>
+        <v>3379</v>
       </c>
       <c r="L23" s="39">
         <v>10</v>
@@ -59469,13 +59472,13 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>3379</v>
+        <v>3380</v>
       </c>
       <c r="B24" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D24" t="s">
         <v>355</v>
@@ -59484,10 +59487,10 @@
         <v>70</v>
       </c>
       <c r="F24" s="35" t="s">
-        <v>3376</v>
+        <v>3377</v>
       </c>
       <c r="G24" s="35" t="s">
-        <v>3377</v>
+        <v>3378</v>
       </c>
       <c r="H24" s="38">
         <v>1000</v>
@@ -59499,7 +59502,7 @@
         <v>1</v>
       </c>
       <c r="K24" s="39" t="s">
-        <v>3379</v>
+        <v>3380</v>
       </c>
       <c r="L24" s="39">
         <v>10</v>
@@ -59552,13 +59555,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>3380</v>
+        <v>3381</v>
       </c>
       <c r="B25" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C25" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D25" t="s">
         <v>355</v>
@@ -59567,10 +59570,10 @@
         <v>70</v>
       </c>
       <c r="F25" s="35" t="s">
-        <v>3376</v>
+        <v>3377</v>
       </c>
       <c r="G25" s="35" t="s">
-        <v>3377</v>
+        <v>3378</v>
       </c>
       <c r="H25" s="38">
         <v>1000</v>
@@ -59582,7 +59585,7 @@
         <v>1</v>
       </c>
       <c r="K25" s="39" t="s">
-        <v>3380</v>
+        <v>3381</v>
       </c>
       <c r="L25" s="39">
         <v>10</v>
@@ -59635,13 +59638,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>3381</v>
+        <v>3382</v>
       </c>
       <c r="B26" t="s">
-        <v>3368</v>
+        <v>3369</v>
       </c>
       <c r="C26" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D26" t="s">
         <v>355</v>
@@ -59650,10 +59653,10 @@
         <v>70</v>
       </c>
       <c r="F26" s="35" t="s">
-        <v>3376</v>
+        <v>3377</v>
       </c>
       <c r="G26" s="35" t="s">
-        <v>3377</v>
+        <v>3378</v>
       </c>
       <c r="H26" s="38">
         <v>1000</v>
@@ -59665,7 +59668,7 @@
         <v>1</v>
       </c>
       <c r="K26" s="39" t="s">
-        <v>3381</v>
+        <v>3382</v>
       </c>
       <c r="L26" s="39">
         <v>10</v>
@@ -68279,13 +68282,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3382</v>
+        <v>3383</v>
       </c>
       <c r="B2" t="s">
-        <v>3383</v>
+        <v>3384</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D2" t="s">
         <v>2871</v>
@@ -68294,10 +68297,10 @@
         <v>70</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>3384</v>
+        <v>3385</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3385</v>
+        <v>3386</v>
       </c>
       <c r="H2" s="38">
         <v>900</v>
@@ -68309,7 +68312,7 @@
         <v>2</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3382</v>
+        <v>3383</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -68359,13 +68362,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3386</v>
+        <v>3387</v>
       </c>
       <c r="B3" t="s">
-        <v>3383</v>
+        <v>3384</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D3" t="s">
         <v>2871</v>
@@ -68374,10 +68377,10 @@
         <v>70</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>3384</v>
+        <v>3385</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3385</v>
+        <v>3386</v>
       </c>
       <c r="H3" s="38">
         <v>900</v>
@@ -68389,7 +68392,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3386</v>
+        <v>3387</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -68439,13 +68442,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3387</v>
+        <v>3388</v>
       </c>
       <c r="B4" t="s">
-        <v>3383</v>
+        <v>3384</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D4" t="s">
         <v>2871</v>
@@ -68454,10 +68457,10 @@
         <v>70</v>
       </c>
       <c r="F4" s="35" t="s">
-        <v>3384</v>
+        <v>3385</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3385</v>
+        <v>3386</v>
       </c>
       <c r="H4" s="38">
         <v>900</v>
@@ -68469,7 +68472,7 @@
         <v>2</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3387</v>
+        <v>3388</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -68519,13 +68522,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3388</v>
+        <v>3389</v>
       </c>
       <c r="B5" t="s">
-        <v>3383</v>
+        <v>3384</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D5" t="s">
         <v>2871</v>
@@ -68534,10 +68537,10 @@
         <v>70</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>3384</v>
+        <v>3385</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3385</v>
+        <v>3386</v>
       </c>
       <c r="H5" s="38">
         <v>900</v>
@@ -68549,7 +68552,7 @@
         <v>2</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3388</v>
+        <v>3389</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -68599,13 +68602,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3389</v>
+        <v>3390</v>
       </c>
       <c r="B6" t="s">
-        <v>3383</v>
+        <v>3384</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D6" t="s">
         <v>2871</v>
@@ -68614,10 +68617,10 @@
         <v>70</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>3384</v>
+        <v>3385</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3385</v>
+        <v>3386</v>
       </c>
       <c r="H6" s="38">
         <v>900</v>
@@ -68629,7 +68632,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3389</v>
+        <v>3390</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -68679,13 +68682,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>3390</v>
+        <v>3391</v>
       </c>
       <c r="B7" t="s">
-        <v>3383</v>
+        <v>3384</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D7" t="s">
         <v>2871</v>
@@ -68694,10 +68697,10 @@
         <v>70</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>3384</v>
+        <v>3385</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3385</v>
+        <v>3386</v>
       </c>
       <c r="H7" s="38">
         <v>900</v>
@@ -68709,7 +68712,7 @@
         <v>2</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3390</v>
+        <v>3391</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -68759,13 +68762,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3391</v>
+        <v>3392</v>
       </c>
       <c r="B8" t="s">
-        <v>3392</v>
+        <v>3393</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D8" t="s">
         <v>2871</v>
@@ -68777,7 +68780,7 @@
         <v>341</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3393</v>
+        <v>3394</v>
       </c>
       <c r="H8" s="38">
         <v>900</v>
@@ -68789,7 +68792,7 @@
         <v>2</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3391</v>
+        <v>3392</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -68828,7 +68831,7 @@
         <v>78</v>
       </c>
       <c r="BA8" t="s">
-        <v>3394</v>
+        <v>3395</v>
       </c>
       <c r="BC8" t="s">
         <v>172</v>
@@ -68839,13 +68842,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>3395</v>
+        <v>3396</v>
       </c>
       <c r="B9" t="s">
-        <v>3392</v>
+        <v>3393</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D9" t="s">
         <v>2871</v>
@@ -68857,7 +68860,7 @@
         <v>341</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3393</v>
+        <v>3394</v>
       </c>
       <c r="H9" s="38">
         <v>900</v>
@@ -68869,7 +68872,7 @@
         <v>2</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3395</v>
+        <v>3396</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -68908,7 +68911,7 @@
         <v>78</v>
       </c>
       <c r="BA9" t="s">
-        <v>3394</v>
+        <v>3395</v>
       </c>
       <c r="BC9" t="s">
         <v>172</v>
@@ -68919,13 +68922,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>3396</v>
+        <v>3397</v>
       </c>
       <c r="B10" t="s">
-        <v>3392</v>
+        <v>3393</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D10" t="s">
         <v>2871</v>
@@ -68937,7 +68940,7 @@
         <v>341</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>3393</v>
+        <v>3394</v>
       </c>
       <c r="H10" s="38">
         <v>900</v>
@@ -68949,7 +68952,7 @@
         <v>2</v>
       </c>
       <c r="K10" s="39" t="s">
-        <v>3396</v>
+        <v>3397</v>
       </c>
       <c r="L10" s="39">
         <v>10</v>
@@ -68988,7 +68991,7 @@
         <v>78</v>
       </c>
       <c r="BA10" t="s">
-        <v>3394</v>
+        <v>3395</v>
       </c>
       <c r="BC10" t="s">
         <v>172</v>
@@ -68999,13 +69002,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>3397</v>
+        <v>3398</v>
       </c>
       <c r="B11" t="s">
-        <v>3392</v>
+        <v>3393</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D11" t="s">
         <v>2871</v>
@@ -69017,7 +69020,7 @@
         <v>341</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>3393</v>
+        <v>3394</v>
       </c>
       <c r="H11" s="38">
         <v>900</v>
@@ -69029,7 +69032,7 @@
         <v>2</v>
       </c>
       <c r="K11" s="39" t="s">
-        <v>3397</v>
+        <v>3398</v>
       </c>
       <c r="L11" s="39">
         <v>10</v>
@@ -69068,7 +69071,7 @@
         <v>78</v>
       </c>
       <c r="BA11" t="s">
-        <v>3394</v>
+        <v>3395</v>
       </c>
       <c r="BC11" t="s">
         <v>172</v>
@@ -69079,13 +69082,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>3398</v>
+        <v>3399</v>
       </c>
       <c r="B12" t="s">
-        <v>3392</v>
+        <v>3393</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D12" t="s">
         <v>2871</v>
@@ -69097,7 +69100,7 @@
         <v>341</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>3393</v>
+        <v>3394</v>
       </c>
       <c r="H12" s="38">
         <v>900</v>
@@ -69109,7 +69112,7 @@
         <v>2</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>3398</v>
+        <v>3399</v>
       </c>
       <c r="L12" s="39">
         <v>10</v>
@@ -69148,7 +69151,7 @@
         <v>78</v>
       </c>
       <c r="BA12" t="s">
-        <v>3394</v>
+        <v>3395</v>
       </c>
       <c r="BC12" t="s">
         <v>172</v>
@@ -69159,13 +69162,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>3399</v>
+        <v>3400</v>
       </c>
       <c r="B13" t="s">
-        <v>3392</v>
+        <v>3393</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>3328</v>
       </c>
       <c r="D13" t="s">
         <v>2871</v>
@@ -69177,7 +69180,7 @@
         <v>341</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>3393</v>
+        <v>3394</v>
       </c>
       <c r="H13" s="38">
         <v>900</v>
@@ -69189,7 +69192,7 @@
         <v>2</v>
       </c>
       <c r="K13" s="39" t="s">
-        <v>3399</v>
+        <v>3400</v>
       </c>
       <c r="L13" s="39">
         <v>10</v>
@@ -69228,7 +69231,7 @@
         <v>78</v>
       </c>
       <c r="BA13" t="s">
-        <v>3394</v>
+        <v>3395</v>
       </c>
       <c r="BC13" t="s">
         <v>172</v>

</xml_diff>